<commit_message>
Completed ReactJS Hands-on 2 - Student Management Portal
</commit_message>
<xml_diff>
--- a/Digital-Nurture-JavaFSE-main/Java FSE/Deepskilling/DN - Java FSE Mandatory hands-on detail.xlsx
+++ b/Digital-Nurture-JavaFSE-main/Java FSE/Deepskilling/DN - Java FSE Mandatory hands-on detail.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cognizantonline-my.sharepoint.com/personal/239914_cognizant_com/Documents/2025/Academy work/Digital Nurture/DN 5.0/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cognizant-Assignments\Digital-Nurture-JavaFSE-main\Java FSE\Deepskilling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{38815D58-CAD9-44C0-B366-FB59C6453CF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A83D4995-9CD0-446A-9BFE-55A9EAB2B518}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF93051B-1D67-433E-924A-B5F8F7AD8797}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E078EC40-2268-4F4F-B14B-9403122955B8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E078EC40-2268-4F4F-B14B-9403122955B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Java FSE" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -475,14 +473,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -495,16 +503,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -840,30 +838,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B57EFDF7-9EDE-4E32-9B50-93240323B319}">
   <dimension ref="A1:E48"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.08984375" customWidth="1"/>
-    <col min="2" max="2" width="22.6328125" customWidth="1"/>
-    <col min="3" max="3" width="47.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.26953125" customWidth="1"/>
-    <col min="5" max="5" width="30.453125" customWidth="1"/>
+    <col min="1" max="1" width="23.109375" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
+    <col min="3" max="3" width="47.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.21875" customWidth="1"/>
+    <col min="5" max="5" width="30.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="13" t="s">
+      <c r="C1" s="16"/>
+      <c r="D1" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="E1" s="14"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="16"/>
+      <c r="E1" s="18"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="10"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -877,7 +875,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
@@ -890,7 +888,7 @@
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
@@ -903,7 +901,7 @@
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
     </row>
-    <row r="5" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>6</v>
       </c>
@@ -916,7 +914,7 @@
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
     </row>
-    <row r="6" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
@@ -929,7 +927,7 @@
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
@@ -942,7 +940,7 @@
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
@@ -955,7 +953,7 @@
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
     </row>
-    <row r="9" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
@@ -968,7 +966,7 @@
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
     </row>
-    <row r="10" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
@@ -981,29 +979,29 @@
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
     </row>
-    <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A11" s="9" t="s">
+    <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="13" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="10"/>
-      <c r="B12" s="8"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="12"/>
+      <c r="B12" s="14"/>
       <c r="C12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-    </row>
-    <row r="13" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+    </row>
+    <row r="13" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>14</v>
       </c>
@@ -1016,7 +1014,7 @@
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>14</v>
       </c>
@@ -1029,7 +1027,7 @@
       <c r="D14" s="4"/>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>23</v>
       </c>
@@ -1042,7 +1040,7 @@
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>26</v>
       </c>
@@ -1057,7 +1055,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>26</v>
       </c>
@@ -1072,7 +1070,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>26</v>
       </c>
@@ -1087,7 +1085,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>34</v>
       </c>
@@ -1104,7 +1102,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>34</v>
       </c>
@@ -1121,7 +1119,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>34</v>
       </c>
@@ -1134,7 +1132,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>34</v>
       </c>
@@ -1147,7 +1145,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>34</v>
       </c>
@@ -1160,7 +1158,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>34</v>
       </c>
@@ -1173,7 +1171,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>46</v>
       </c>
@@ -1190,7 +1188,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>46</v>
       </c>
@@ -1203,7 +1201,7 @@
       <c r="D26" s="4"/>
       <c r="E26" s="4"/>
     </row>
-    <row r="27" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>46</v>
       </c>
@@ -1216,7 +1214,7 @@
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
     </row>
-    <row r="28" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>46</v>
       </c>
@@ -1229,7 +1227,7 @@
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
     </row>
-    <row r="29" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>46</v>
       </c>
@@ -1242,7 +1240,7 @@
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
     </row>
-    <row r="30" spans="1:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>46</v>
       </c>
@@ -1255,33 +1253,33 @@
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
     </row>
-    <row r="31" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A31" s="9" t="s">
+    <row r="31" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="D31" s="9" t="s">
+      <c r="D31" s="11" t="s">
         <v>59</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="10"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="10"/>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="12"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="12"/>
       <c r="E32" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>63</v>
       </c>
@@ -1298,7 +1296,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>63</v>
       </c>
@@ -1315,7 +1313,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>63</v>
       </c>
@@ -1332,7 +1330,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>63</v>
       </c>
@@ -1345,7 +1343,7 @@
       <c r="D36" s="4"/>
       <c r="E36" s="4"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>63</v>
       </c>
@@ -1358,7 +1356,7 @@
       <c r="D37" s="4"/>
       <c r="E37" s="4"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>63</v>
       </c>
@@ -1375,7 +1373,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>63</v>
       </c>
@@ -1392,7 +1390,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>63</v>
       </c>
@@ -1409,7 +1407,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>63</v>
       </c>
@@ -1426,7 +1424,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>63</v>
       </c>
@@ -1443,7 +1441,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>82</v>
       </c>
@@ -1456,7 +1454,7 @@
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>82</v>
       </c>
@@ -1469,7 +1467,7 @@
       <c r="D44" s="4"/>
       <c r="E44" s="4"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>82</v>
       </c>
@@ -1482,7 +1480,7 @@
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>82</v>
       </c>
@@ -1495,7 +1493,7 @@
       <c r="D46" s="4"/>
       <c r="E46" s="4"/>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>82</v>
       </c>
@@ -1508,18 +1506,18 @@
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="17" t="s">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B48" s="18" t="s">
+      <c r="B48" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="C48" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="D48" s="18"/>
-      <c r="E48" s="18"/>
+      <c r="C48" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1540,6 +1538,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="c6f516c4-2602-422c-aa9a-755893ba4f98">
@@ -1548,15 +1555,6 @@
     <TaxCatchAll xmlns="3c35e321-f73a-4dae-ae38-a0459de24735"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1820,6 +1818,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F0F638-0648-46BA-B1DF-3E4F6ADB00E4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19B84191-BBE7-412A-A5F6-7B8D27AECA6C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -1833,14 +1839,6 @@
     <ds:schemaRef ds:uri="951c5514-b77c-4532-82d5-a05f2f7d58e2"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15F0F638-0648-46BA-B1DF-3E4F6ADB00E4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>